<commit_message>
renewal fixes,e2e fixes and dlg 2.0 journey added
</commit_message>
<xml_diff>
--- a/data/application_data.xlsx
+++ b/data/application_data.xlsx
@@ -502,17 +502,14 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v/>
+        <v>8108556733</v>
       </c>
       <c r="B2" t="str">
-        <v>masira darvesh</v>
+        <v>masira</v>
       </c>
       <c r="C2" t="str">
         <v>Bangalore (Whitefield)</v>
       </c>
-      <c r="D2" t="str">
-        <v>BA Photography</v>
-      </c>
       <c r="E2" t="str">
         <v>-2023</v>
       </c>
@@ -535,7 +532,7 @@
         <v>76000</v>
       </c>
       <c r="L2" t="str">
-        <v>Student+Parent/Guardian</v>
+        <v>Student</v>
       </c>
       <c r="M2" t="str">
         <v>ahmed</v>
@@ -603,7 +600,7 @@
     </row>
     <row r="3">
       <c r="A3" t="str">
-        <v/>
+        <v>8108556708</v>
       </c>
       <c r="B3" t="str">
         <v>masira darvesh</v>
@@ -645,7 +642,7 @@
         <v>parent</v>
       </c>
       <c r="O3" t="str">
-        <v>ABCDE1234F</v>
+        <v>DDDPD1621M</v>
       </c>
       <c r="P3" t="str">
         <v>Male</v>
@@ -660,7 +657,7 @@
         <v>15</v>
       </c>
       <c r="T3" t="str">
-        <v>Single</v>
+        <v>Divorced</v>
       </c>
       <c r="U3" t="str">
         <v>test.parent@example.com</v>

</xml_diff>